<commit_message>
did a LOT of refactoring
</commit_message>
<xml_diff>
--- a/chemical_database.xlsx
+++ b/chemical_database.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="59">
   <si>
     <t>Searched Chemical Name</t>
   </si>
@@ -35,6 +35,9 @@
     <t>SDS Link</t>
   </si>
   <si>
+    <t>Storage Notes</t>
+  </si>
+  <si>
     <t>SDS Revision Date</t>
   </si>
   <si>
@@ -92,7 +95,7 @@
     <t>Pictogram Codes (for export)</t>
   </si>
   <si>
-    <t>SDS DOT Class (fix later)</t>
+    <t>Generated Classification (Class)</t>
   </si>
   <si>
     <t>PubChem CID Number</t>
@@ -144,7 +147,7 @@
       <rPr>
         <b/>
       </rPr>
-      <t>Barium nitrate</t>
+      <t>N/A</t>
     </r>
     <r>
       <t xml:space="preserve">
@@ -248,6 +251,9 @@
   </si>
   <si>
     <t>https://www.fishersci.com/store/msds?partNumber=AC192555000&amp;productDescription=barium-nitrate-acs-reag-kg&amp;vendorId=VN00032119&amp;keyword=true&amp;countryCode=US&amp;language=en</t>
+  </si>
+  <si>
+    <t>Keep containers tightly closed in a dry, cool and well-ventilated place. Do not store near combustible materials. Incompatible Materials. Organic materials. Acids. Bases. Acid anhydrides. Metals. Reducing Agent. Strong reducing agents. Combustible material.</t>
   </si>
   <si>
     <t>24-Dec-2021</t>
@@ -280,7 +286,7 @@
   <si>
     <t xml:space="preserve">May intensify fire; oxidizer Toxic if swallowed 
 Causes serious eye irritation 
-Harmful if inhaled Company Fisher Scientific Company One Reagent Lane Fair Lawn, NJ 07410 Tel: (201) 796-7100 Acros Organics One Reagent Lane Fair Lawn, NJ 07410 Acute oral toxicity Category 3 Acute Inhalation Toxicity - Dusts and Mists Category 4 Serious Eye Damage/Eye Irritation Category 2 Oxidizing solids Category 2</t>
+Harmful if inhaled 0 Acute oral toxicity Category 3 Acute Inhalation Toxicity - Dusts and Mists Category 4 Serious Eye Damage/Eye Irritation Category 2 Oxidizing solids Category 2</t>
   </si>
   <si>
     <t xml:space="preserve">H272 (68.7%): May intensify fire; oxidizer [Danger Oxidizing liquids; Oxidizing solids]
@@ -302,16 +308,13 @@
 Health Hazard</t>
   </si>
   <si>
-    <t>temp</t>
-  </si>
-  <si>
-    <t>5.1</t>
+    <t>Inorganic salt</t>
   </si>
   <si>
     <t>EM Science</t>
   </si>
   <si>
-    <t>500 g</t>
+    <t>g</t>
   </si>
   <si>
     <t>6-144</t>
@@ -744,7 +747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AQ2"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
@@ -753,46 +756,46 @@
     <col min="4" max="4" width="24" style="1" customWidth="1"/>
     <col min="5" max="5" width="22" style="1" customWidth="1"/>
     <col min="6" max="6" width="90" style="1" customWidth="1"/>
-    <col min="7" max="7" width="100" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2" style="1" customWidth="1"/>
-    <col min="11" max="11" width="24" style="1" customWidth="1"/>
-    <col min="12" max="12" width="19" style="1" customWidth="1"/>
-    <col min="13" max="13" width="23" style="1" customWidth="1"/>
-    <col min="14" max="14" width="2" style="1" customWidth="1"/>
-    <col min="15" max="15" width="21" style="1" customWidth="1"/>
-    <col min="16" max="16" width="16" style="1" customWidth="1"/>
-    <col min="17" max="17" width="24" style="1" customWidth="1"/>
-    <col min="18" max="18" width="2" style="1" customWidth="1"/>
-    <col min="19" max="19" width="45" style="1" customWidth="1"/>
-    <col min="20" max="20" width="88" style="1" customWidth="1"/>
-    <col min="21" max="21" width="2" style="1" customWidth="1"/>
-    <col min="22" max="22" width="23" style="1" customWidth="1"/>
-    <col min="23" max="23" width="27" style="1" customWidth="1"/>
-    <col min="24" max="24" width="2" style="1" customWidth="1"/>
-    <col min="25" max="25" width="22" style="1" customWidth="1"/>
-    <col min="26" max="26" width="26" style="1" customWidth="1"/>
-    <col min="27" max="27" width="2" style="1" customWidth="1"/>
-    <col min="28" max="28" width="17" style="1" customWidth="1"/>
-    <col min="29" max="29" width="21" style="1" customWidth="1"/>
-    <col min="30" max="30" width="2" style="1" customWidth="1"/>
-    <col min="31" max="31" width="100" style="1" customWidth="1"/>
-    <col min="32" max="32" width="100" style="2" customWidth="1"/>
-    <col min="33" max="33" width="45" style="1" customWidth="1"/>
-    <col min="34" max="34" width="30" style="1" customWidth="1"/>
-    <col min="35" max="35" width="27" style="1" customWidth="1"/>
-    <col min="36" max="36" width="2" style="1" customWidth="1"/>
-    <col min="37" max="37" width="20" style="1" customWidth="1"/>
-    <col min="38" max="38" width="12" style="1" customWidth="1"/>
-    <col min="39" max="39" width="10" style="1" customWidth="1"/>
-    <col min="40" max="40" width="7" style="1" customWidth="1"/>
-    <col min="41" max="41" width="10" style="1" customWidth="1"/>
-    <col min="42" max="42" width="9" style="1" customWidth="1"/>
-    <col min="43" max="43" width="15" style="1" customWidth="1"/>
+    <col min="7" max="8" width="100" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8" style="1" customWidth="1"/>
+    <col min="11" max="11" width="2" style="1" customWidth="1"/>
+    <col min="12" max="12" width="24" style="1" customWidth="1"/>
+    <col min="13" max="13" width="19" style="1" customWidth="1"/>
+    <col min="14" max="14" width="23" style="1" customWidth="1"/>
+    <col min="15" max="15" width="2" style="1" customWidth="1"/>
+    <col min="16" max="16" width="21" style="1" customWidth="1"/>
+    <col min="17" max="17" width="16" style="1" customWidth="1"/>
+    <col min="18" max="18" width="24" style="1" customWidth="1"/>
+    <col min="19" max="19" width="2" style="1" customWidth="1"/>
+    <col min="20" max="20" width="45" style="1" customWidth="1"/>
+    <col min="21" max="21" width="88" style="1" customWidth="1"/>
+    <col min="22" max="22" width="2" style="1" customWidth="1"/>
+    <col min="23" max="23" width="23" style="1" customWidth="1"/>
+    <col min="24" max="24" width="27" style="1" customWidth="1"/>
+    <col min="25" max="25" width="2" style="1" customWidth="1"/>
+    <col min="26" max="26" width="22" style="1" customWidth="1"/>
+    <col min="27" max="27" width="26" style="1" customWidth="1"/>
+    <col min="28" max="28" width="2" style="1" customWidth="1"/>
+    <col min="29" max="29" width="17" style="1" customWidth="1"/>
+    <col min="30" max="30" width="21" style="1" customWidth="1"/>
+    <col min="31" max="31" width="2" style="1" customWidth="1"/>
+    <col min="32" max="32" width="100" style="1" customWidth="1"/>
+    <col min="33" max="33" width="100" style="2" customWidth="1"/>
+    <col min="34" max="34" width="45" style="1" customWidth="1"/>
+    <col min="35" max="35" width="30" style="1" customWidth="1"/>
+    <col min="36" max="36" width="34" style="1" customWidth="1"/>
+    <col min="37" max="37" width="2" style="1" customWidth="1"/>
+    <col min="38" max="38" width="20" style="1" customWidth="1"/>
+    <col min="39" max="39" width="12" style="1" customWidth="1"/>
+    <col min="40" max="40" width="10" style="1" customWidth="1"/>
+    <col min="41" max="41" width="7" style="1" customWidth="1"/>
+    <col min="42" max="42" width="10" style="1" customWidth="1"/>
+    <col min="43" max="43" width="9" style="1" customWidth="1"/>
+    <col min="44" max="44" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -820,76 +823,76 @@
       <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>0</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>10</v>
       </c>
       <c r="M1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" s="4" t="s">
+      <c r="N1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>1</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>12</v>
       </c>
       <c r="Q1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="S1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>14</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="V1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>16</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="W1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="X1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>18</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="Z1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AB1" s="4" t="s">
+      <c r="AA1" s="4" t="s">
         <v>20</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="AC1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="AD1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AD1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AE1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="AG1" s="4" t="s">
+      <c r="AG1" s="6" t="s">
         <v>24</v>
       </c>
       <c r="AH1" s="4" t="s">
@@ -898,11 +901,11 @@
       <c r="AI1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AJ1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK1" s="4" t="s">
+      <c r="AJ1" s="4" t="s">
         <v>27</v>
+      </c>
+      <c r="AK1" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="AL1" s="4" t="s">
         <v>28</v>
@@ -922,127 +925,130 @@
       <c r="AQ1" s="4" t="s">
         <v>33</v>
       </c>
+      <c r="AR1" s="4" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" s="7">
         <v>90</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="7" t="s">
         <v>35</v>
       </c>
+      <c r="N2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="P2" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>42</v>
+        <v>36</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="T2" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="V2" s="7" t="s">
         <v>44</v>
       </c>
+      <c r="U2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="W2" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="X2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y2" s="7" t="s">
         <v>46</v>
       </c>
+      <c r="X2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="Z2" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="AA2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AB2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="AA2" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="AC2" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AD2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE2" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF2" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="AG2" s="7" t="s">
+      <c r="AD2" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF2" s="7" t="s">
         <v>50</v>
       </c>
+      <c r="AG2" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="AH2" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AI2" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="AJ2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK2" s="7">
+        <v>10</v>
+      </c>
+      <c r="AJ2" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL2" s="7">
         <v>24798</v>
-      </c>
-      <c r="AL2" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="AM2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="AN2" s="7" t="s">
-        <v>9</v>
+      <c r="AN2" s="7">
+        <v>500</v>
       </c>
       <c r="AO2" s="7" t="s">
         <v>55</v>
@@ -1052,6 +1058,9 @@
       </c>
       <c r="AQ2" s="7" t="s">
         <v>57</v>
+      </c>
+      <c r="AR2" s="7" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>